<commit_message>
fix fixcal and change postcard play
</commit_message>
<xml_diff>
--- a/2025GoldenDolphin/Assets/Editor/Data.xlsx
+++ b/2025GoldenDolphin/Assets/Editor/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\系统\文档\GitHub\2025GoldenDolphin\2025GoldenDolphin\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A70BB7F-4C70-42D6-85A3-5C41AB24026A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6993F4EB-3474-48AD-B7C4-08B500C7BD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BasicItemData" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="135">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -356,6 +356,171 @@
   </si>
   <si>
     <t>bagHSpritePath</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>texturePath</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>textContent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>scale</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>failed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>roundStaEff</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>roundEndEff</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>留空字段，表示回合开始效果的字典的key</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2b-book-pinecone.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2b-book-trash.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2b-chocolate-trash.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2b-collar-chocolate.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2b-postcard-pinecone.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2g-book-collar.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2g-book-postcard.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2g-pinecone-collar.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2g-pinecone-trash.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/2g-postcard-chocolate.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/3b-book-pinecone-postcard.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/3b-book-trash-postcard.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/3b-collar-pinecone-trash.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/3g-book-pinecone-collar.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/3g-chocolate-book-postcard.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/3g-chocolate-trash-collar.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Assets/Resources/Images/Postcard/failed.png</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我早该知道的。</t>
+  </si>
+  <si>
+    <t>朋友转学了，久违的约我在公园见最后一面。</t>
+  </si>
+  <si>
+    <t>我失约了，我和朋友就这样吵架了。</t>
+  </si>
+  <si>
+    <t>小白走了。我把它埋在了我们相遇的地方。</t>
+  </si>
+  <si>
+    <t>终于毕业了，未来会像巧克力一样美好吗？</t>
+  </si>
+  <si>
+    <t>成功制止小白偷吃巧克力，大胜利！</t>
+  </si>
+  <si>
+    <t>一张失焦的拍立得。</t>
+  </si>
+  <si>
+    <t>撞到期中考试，没能和朋友告别，我又失约了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>坐到垃圾桶旁边了，真讨厌啊。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小白偷吃巧克力进了医院，好自责。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>偷偷把小白带去了教室，它很乖，上课的时候没有叫，老师没有发现。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>生日的时候朋友给我写了明信片。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>朋友走后去公园赴失约的约，捡到了小白，我不再是一个人了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>和朋友去公园捡落叶，我们最喜欢这里了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>终于告诉他我的心意了，他收下了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我和朋友太不同了，也许这是注定的结局。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>逃课带小白去公园，我们也最喜欢这里了。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1.6,1,1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1,1.6,1)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -399,10 +564,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -890,16 +1061,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE023639-9E85-44E8-8C62-DC543CB666CF}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="28" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.77734375" customWidth="1"/>
+    <col min="7" max="7" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -913,231 +1089,416 @@
         <v>56</v>
       </c>
       <c r="E1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I1" t="s">
+        <v>97</v>
+      </c>
+      <c r="J1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="2">
         <v>3</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="E2" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>3</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="E3" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>4</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="E4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="2">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="E5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="2">
         <v>4</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="E6" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="2">
         <v>3</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="E7" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="2">
         <v>3</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="E8" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="2">
         <v>4</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="E9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="2">
         <v>4</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="E10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="2">
         <v>4</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="E11" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="2">
         <v>5</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="E12" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="2">
         <v>5</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="E13" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="2">
         <v>6</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="E14" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="2">
         <v>5</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="E15" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="2">
         <v>5</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="E16" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="2">
         <v>6</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="2">
         <v>0</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="2">
+        <v>0</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>